<commit_message>
Datasets de MP sin la lista de trampas («Sembrados») en el LÉAME ni en el brief
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datasets/mp/01 Ventas por campaña y referencia - sintético.xlsx
+++ b/datasets/mp/01 Ventas por campaña y referencia - sintético.xlsx
@@ -26654,27 +26654,9 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Sembrados a propósito: una referencia de calzado con devoluciones que se disparan desde C06; una referencia de lencería con devolución alta por talla;</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>efecto de temporada (Día de la Madre, Día del Padre, Regreso a clases). Errores de datos: una categoría mal escrita,</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>una fila con más devoluciones que unidades y una fila duplicada. Que la IA los encuentre antes de concluir.</t>
-        </is>
-      </c>
-    </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>